<commit_message>
Add backbone/inference latency, trade-off figure, richer results.xlsx, F01uncal predictions; regrade I5 at 288
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submissions/2A202602796-HoDangPhuc/results.xlsx
+++ b/submissions/2A202602796-HoDangPhuc/results.xlsx
@@ -15,6 +15,8 @@
     <sheet name="PerClass" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Latency" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Summary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Latency_extra" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Final_vs_baseline" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,12 +38,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -62,11 +74,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X8"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,6 +570,26 @@
           <t>gpu</t>
         </is>
       </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>lat_p50_ms_b1_fp32</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>lat_p95_ms_b1_fp32</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>lat_p99_ms_b1_fp32</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>lat_p50_ms_b1_fp16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -610,14 +644,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="n">
         <v>0.0001</v>
       </c>
@@ -642,6 +673,18 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="Y2" t="n">
+        <v>5.6692</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>8.4031</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>8.430899999999999</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>6.4085</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -696,14 +739,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
         <v>0.0001</v>
       </c>
@@ -728,6 +768,18 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="Y3" t="n">
+        <v>7.7003</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>8.386200000000001</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>10.0123</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>6.6366</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -782,14 +834,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
         <v>0.0001</v>
       </c>
@@ -814,6 +863,18 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="Y4" t="n">
+        <v>5.3467</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>9.3529</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>9.3673</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>5.3158</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -868,14 +929,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
       <c r="S5" t="n">
         <v>0.0001</v>
       </c>
@@ -900,6 +958,18 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="Y5" t="n">
+        <v>4.5783</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>4.912</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>5.0987</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>4.3708</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -954,14 +1024,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
         <v>0.0001</v>
       </c>
@@ -986,6 +1053,18 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="Y6" t="n">
+        <v>9.4582</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>12.7651</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>10.2475</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1040,14 +1119,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
         <v>0.0001</v>
       </c>
@@ -1072,6 +1148,18 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="Y7" t="n">
+        <v>7.7865</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>8.6873</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>8.7674</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1126,14 +1214,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
         <v>0.0001</v>
       </c>
@@ -1157,6 +1242,109 @@
         <is>
           <t>Tesla T4</t>
         </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>5.9894</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>6.5658</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>6.9726</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>7.2187</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>cấu hình</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_test (3 seed)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>top1_test</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ece_test</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>p95_ms_b1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C00 mốc (ConvNeXt-T, 1-view 224)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.9692 ± 0.0024</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.9760 ± 0.0017</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.0136 ± 0.0012</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>9.359299999999999</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>F01 tốt nhất (C13 + res288 + TS)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>0.9774 ± 0.0006</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0.9812 ± 0.0005</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>0.0041 ± 0.0013</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>9.368499999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1353,14 +1541,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="n">
         <v>0.0001</v>
       </c>
@@ -1442,14 +1627,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
         <v>0.0001</v>
       </c>
@@ -1531,14 +1713,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
         <v>0.0001</v>
       </c>
@@ -1620,14 +1799,11 @@
           <t>color</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
       <c r="S5" t="n">
         <v>0.0001</v>
       </c>
@@ -1709,14 +1885,11 @@
           <t>trivial</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
         <v>0.0001</v>
       </c>
@@ -1808,8 +1981,6 @@
           <t>ce</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
         <v>0.0001</v>
       </c>
@@ -1901,8 +2072,6 @@
           <t>ce</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
         <v>0.0001</v>
       </c>
@@ -1984,14 +2153,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
         <v>0.0001</v>
       </c>
@@ -2073,14 +2239,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>focal</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
         <v>0.0001</v>
       </c>
@@ -2162,14 +2325,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>ce_weighted</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
         <v>0.0001</v>
       </c>
@@ -2251,7 +2411,6 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>ce</t>
@@ -2262,7 +2421,6 @@
           <t>balanced</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="n">
         <v>0.0001</v>
       </c>
@@ -2344,13 +2502,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="n">
         <v>0.995</v>
       </c>
@@ -2435,14 +2591,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
       <c r="S14" t="n">
         <v>0.0002</v>
       </c>
@@ -2534,8 +2687,6 @@
           <t>ce_weighted</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
         <v>0.0001</v>
       </c>
@@ -2753,14 +2904,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="n">
         <v>0.0001</v>
       </c>
@@ -2839,14 +2987,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="n">
         <v>0.0001</v>
       </c>
@@ -2925,14 +3070,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
         <v>0.0001</v>
       </c>
@@ -3011,14 +3153,11 @@
           <t>color</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
       <c r="S5" t="n">
         <v>0.0001</v>
       </c>
@@ -3097,14 +3236,11 @@
           <t>trivial</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
         <v>0.0001</v>
       </c>
@@ -3193,8 +3329,6 @@
           <t>ce</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
         <v>0.0001</v>
       </c>
@@ -3283,8 +3417,6 @@
           <t>ce</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
         <v>0.0001</v>
       </c>
@@ -3363,14 +3495,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
         <v>0.0001</v>
       </c>
@@ -3449,14 +3578,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>focal</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
         <v>0.0001</v>
       </c>
@@ -3535,14 +3661,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>ce_weighted</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
         <v>0.0001</v>
       </c>
@@ -3621,7 +3744,6 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>ce</t>
@@ -3632,7 +3754,6 @@
           <t>balanced</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="n">
         <v>0.0001</v>
       </c>
@@ -3711,13 +3832,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="n">
         <v>0.995</v>
       </c>
@@ -3799,14 +3918,11 @@
           <t>basic</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>ce</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
       <c r="S14" t="n">
         <v>0.0001</v>
       </c>
@@ -3843,7 +3959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3859,27 +3975,47 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>space</t>
+          <t>K</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>macro_f1_val</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>macro_f1_val</t>
+          <t>top1_val</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>top1_val</t>
+          <t>ece_val</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ece_val</t>
+          <t>lat_p50_ms</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>lat_p95_ms</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>lat_p99_ms</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>cost_vs_I00</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ghi_chú</t>
         </is>
       </c>
     </row>
@@ -3894,399 +4030,356 @@
           <t>I00 1-view</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
+      <c r="C2" t="n">
+        <v>1</v>
       </c>
       <c r="D2" t="n">
+        <v>0.9721</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5.4302</v>
+      </c>
+      <c r="H2" t="n">
+        <v>9.359299999999999</v>
+      </c>
+      <c r="I2" t="n">
+        <v>9.3932</v>
+      </c>
+      <c r="J2" t="n">
         <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.9721</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.9789</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.0129</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>I00</t>
+          <t>I01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>I00 1-view</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>logit</t>
-        </is>
+          <t>I01 flip</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0.9717</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9721</v>
+        <v>0.9786</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9789</v>
+        <v>0.0137</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0129</v>
+        <v>8.382999999999999</v>
+      </c>
+      <c r="H3" t="n">
+        <v>11.3782</v>
+      </c>
+      <c r="I3" t="n">
+        <v>11.3972</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1.5438</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>I01</t>
+          <t>I02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>I01 flip</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
+          <t>I02 5crop192</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>0.9695</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9717</v>
+        <v>0.9762999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9786</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.0137</v>
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>chưa đo độ trễ (K=5, F1 không hơn I00)</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>I01</t>
+          <t>I02b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>I01 flip</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>logit</t>
-        </is>
+          <t>I02b 5crop+flip192</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>0.9703000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9715</v>
+        <v>0.9766</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9786</v>
+        <v>0.0081</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0122</v>
+        <v>27.6541</v>
+      </c>
+      <c r="H5" t="n">
+        <v>28.3249</v>
+      </c>
+      <c r="I5" t="n">
+        <v>28.3779</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5.0926</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>I02</t>
+          <t>I04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>I02 5crop192</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
+          <t>res224</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
       </c>
       <c r="D6" t="n">
+        <v>0.9721</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5.4302</v>
+      </c>
+      <c r="H6" t="n">
+        <v>9.359299999999999</v>
+      </c>
+      <c r="I6" t="n">
+        <v>9.3932</v>
+      </c>
+      <c r="J6" t="n">
         <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.9695</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.9762999999999999</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.009599999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>I02</t>
+          <t>I04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>I02 5crop192</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>logit</t>
-        </is>
+          <t>res256</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0.9756</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9695</v>
+        <v>0.9817</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9762999999999999</v>
+        <v>0.0197</v>
       </c>
       <c r="G7" t="n">
-        <v>0.009599999999999999</v>
+        <v>5.7254</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10.4001</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10.4253</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.0544</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>I02b</t>
+          <t>I04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>I02b 5crop+flip192</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
+          <t>res288</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0.9776</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9703000000000001</v>
+        <v>0.9826</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9766</v>
+        <v>0.0299</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0081</v>
+        <v>6.9092</v>
+      </c>
+      <c r="H8" t="n">
+        <v>9.368499999999999</v>
+      </c>
+      <c r="I8" t="n">
+        <v>9.400399999999999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1.2724</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>I02b</t>
+          <t>I04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>I02b 5crop+flip192</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>logit</t>
-        </is>
+          <t>res320</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>0.9777</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9703000000000001</v>
+        <v>0.982</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9766</v>
+        <v>0.0381</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0081</v>
+        <v>8.593500000000001</v>
+      </c>
+      <c r="H9" t="n">
+        <v>14.8999</v>
+      </c>
+      <c r="I9" t="n">
+        <v>14.9273</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1.5825</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>I04</t>
+          <t>I07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>res224</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
+          <t>temperature trước (T=0.875)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
       </c>
       <c r="D10" t="n">
+        <v>0.9721</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.0129</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5.4302</v>
+      </c>
+      <c r="H10" t="n">
+        <v>9.359299999999999</v>
+      </c>
+      <c r="I10" t="n">
+        <v>9.3932</v>
+      </c>
+      <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" t="n">
-        <v>0.9721</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.9789</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.0129</v>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>TS: chi phí thêm không đáng kể (một phép chia logit)</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>I04</t>
+          <t>I07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>res256</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
+          <t>temperature sau (T=0.875)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
       </c>
       <c r="D11" t="n">
+        <v>0.9721</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5.4302</v>
+      </c>
+      <c r="H11" t="n">
+        <v>9.359299999999999</v>
+      </c>
+      <c r="I11" t="n">
+        <v>9.3932</v>
+      </c>
+      <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="E11" t="n">
-        <v>0.9756</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.9817</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.0197</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>I04</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>res288</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.9776</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.9826</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.0299</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>I04</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>res320</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.9777</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.0381</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>I07</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>temperature trước (T=0.875)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.9721</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.9789</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.0129</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>I07</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>temperature sau (T=0.875)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>prob</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.9721</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.9789</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.0054</v>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>TS: chi phí thêm không đáng kể (một phép chia logit)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5391,13 +5484,6 @@
       <c r="I2" t="n">
         <v>174.0675</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5433,13 +5519,6 @@
       <c r="I3" t="n">
         <v>128.2731</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5475,13 +5554,6 @@
       <c r="I4" t="n">
         <v>173.3735</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5517,13 +5589,6 @@
       <c r="I5" t="n">
         <v>235.139</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5559,13 +5624,6 @@
       <c r="I6" t="n">
         <v>636.2472</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5601,13 +5659,6 @@
       <c r="I7" t="n">
         <v>791.5318</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5643,13 +5694,6 @@
       <c r="I8" t="n">
         <v>172.5043</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5685,13 +5729,6 @@
       <c r="I9" t="n">
         <v>224.8779</v>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5727,12 +5764,6 @@
       <c r="I10" t="n">
         <v>204.2046</v>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>không</t>
@@ -5750,7 +5781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5814,71 +5845,6 @@
           <t>epochs</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>init</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>aug</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>mix</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>sampler</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>ema_decay</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>lr_backbone</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>lr_head</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>batch_size</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>torch</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>timm</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>gpu</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>delta_vs_C00</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5923,55 +5889,6 @@
       <c r="L2" t="n">
         <v>12</v>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>cutmix</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>ce</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U2" t="n">
-        <v>64</v>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>2.11.0+cu128</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y2" t="n">
-        <v>0.0042</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6016,766 +5933,1447 @@
       <c r="L3" t="n">
         <v>12</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>trivial</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>ce</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U3" t="n">
-        <v>64</v>
-      </c>
-      <c r="V3" t="inlineStr">
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0.9721</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.9789</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>51.3687</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>224</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9717</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9777</v>
+      </c>
+      <c r="F5" t="n">
+        <v>51.9942</v>
+      </c>
+      <c r="G5" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>224</v>
+      </c>
+      <c r="L5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B03_convnext_tiny</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9777</v>
+      </c>
+      <c r="F6" t="n">
+        <v>52.2154</v>
+      </c>
+      <c r="G6" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>224</v>
+      </c>
+      <c r="L6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.9746</v>
+      </c>
+      <c r="F7" t="n">
+        <v>52.6643</v>
+      </c>
+      <c r="G7" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>224</v>
+      </c>
+      <c r="L7" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>C00</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0.9689</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.9746</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>52.1954</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>224</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.9687</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.9757</v>
+      </c>
+      <c r="F9" t="n">
+        <v>51.173</v>
+      </c>
+      <c r="G9" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>224</v>
+      </c>
+      <c r="L9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.9685</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9743000000000001</v>
+      </c>
+      <c r="F10" t="n">
+        <v>52.923</v>
+      </c>
+      <c r="G10" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>224</v>
+      </c>
+      <c r="L10" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.9655</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9729</v>
+      </c>
+      <c r="F11" t="n">
+        <v>52.5088</v>
+      </c>
+      <c r="G11" t="n">
+        <v>27.827</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4.4548</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>in12k_ft_in1k</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>224</v>
+      </c>
+      <c r="L11" t="n">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>nhóm</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gpu</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dtype</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>img_size</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>p50</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>p99</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>images_per_s</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>torch</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>224</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5.6692</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8.4031</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8.430899999999999</v>
+      </c>
+      <c r="J2" t="n">
+        <v>176.3918</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Tesla T4</t>
         </is>
       </c>
-      <c r="Y3" t="n">
-        <v>0.0034</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>224</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6.4085</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6.9055</v>
+      </c>
+      <c r="I3" t="n">
+        <v>7.3047</v>
+      </c>
+      <c r="J3" t="n">
+        <v>156.043</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C13</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>11</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.9721</v>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>resnext50</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>0.9789</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>51.3687</v>
+        <v>224</v>
       </c>
       <c r="G4" t="n">
-        <v>27.827</v>
+        <v>7.7003</v>
       </c>
       <c r="H4" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>224</v>
-      </c>
-      <c r="L4" t="n">
-        <v>12</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>trivial</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>cutmix</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>ce_weighted</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U4" t="n">
-        <v>64</v>
-      </c>
-      <c r="V4" t="inlineStr">
+        <v>8.386200000000001</v>
+      </c>
+      <c r="I4" t="n">
+        <v>10.0123</v>
+      </c>
+      <c r="J4" t="n">
+        <v>129.8657</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y4" t="n">
-        <v>0.0032</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.9717</v>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>resnext50</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>0.9777</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>51.9942</v>
+        <v>224</v>
       </c>
       <c r="G5" t="n">
-        <v>27.827</v>
+        <v>6.6366</v>
       </c>
       <c r="H5" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>224</v>
-      </c>
-      <c r="L5" t="n">
-        <v>12</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>ce_weighted</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U5" t="n">
-        <v>64</v>
-      </c>
-      <c r="V5" t="inlineStr">
+        <v>7.2603</v>
+      </c>
+      <c r="I5" t="n">
+        <v>9.6561</v>
+      </c>
+      <c r="J5" t="n">
+        <v>150.6797</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.0028</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B03_convnext_tiny</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.971</v>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>0.9777</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>52.2154</v>
+        <v>224</v>
       </c>
       <c r="G6" t="n">
-        <v>27.827</v>
+        <v>5.3467</v>
       </c>
       <c r="H6" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>224</v>
-      </c>
-      <c r="L6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>ce</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U6" t="n">
-        <v>64</v>
-      </c>
-      <c r="V6" t="inlineStr">
+        <v>9.3529</v>
+      </c>
+      <c r="I6" t="n">
+        <v>9.3673</v>
+      </c>
+      <c r="J6" t="n">
+        <v>187.0303</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C11</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>12</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.9692</v>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>convnext_tiny</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
       </c>
       <c r="E7" t="n">
-        <v>0.9746</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>52.6643</v>
+        <v>224</v>
       </c>
       <c r="G7" t="n">
-        <v>27.827</v>
+        <v>5.3158</v>
       </c>
       <c r="H7" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>224</v>
-      </c>
-      <c r="L7" t="n">
-        <v>12</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>ce</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U7" t="n">
-        <v>64</v>
-      </c>
-      <c r="V7" t="inlineStr">
+        <v>6.1342</v>
+      </c>
+      <c r="I7" t="n">
+        <v>6.8405</v>
+      </c>
+      <c r="J7" t="n">
+        <v>188.1175</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y7" t="n">
-        <v>0.0003</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C00</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>9</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.9689</v>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>deit_small</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
       </c>
       <c r="E8" t="n">
-        <v>0.9746</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>52.1954</v>
+        <v>224</v>
       </c>
       <c r="G8" t="n">
-        <v>27.827</v>
+        <v>4.5783</v>
       </c>
       <c r="H8" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>224</v>
-      </c>
-      <c r="L8" t="n">
-        <v>12</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>ce</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U8" t="n">
-        <v>64</v>
-      </c>
-      <c r="V8" t="inlineStr">
+        <v>4.912</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5.0987</v>
+      </c>
+      <c r="J8" t="n">
+        <v>218.4214</v>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y8" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C08</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>11</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.9687</v>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>deit_small</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
       </c>
       <c r="E9" t="n">
-        <v>0.9757</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>51.173</v>
+        <v>224</v>
       </c>
       <c r="G9" t="n">
-        <v>27.827</v>
+        <v>4.3708</v>
       </c>
       <c r="H9" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>224</v>
-      </c>
-      <c r="L9" t="n">
-        <v>12</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>focal</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U9" t="n">
-        <v>64</v>
-      </c>
-      <c r="V9" t="inlineStr">
+        <v>4.7818</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5.3527</v>
+      </c>
+      <c r="J9" t="n">
+        <v>228.7902</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y9" t="n">
-        <v>-0.0002</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C07</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.9685</v>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>swin_tiny</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
       </c>
       <c r="E10" t="n">
-        <v>0.9743000000000001</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>52.923</v>
+        <v>224</v>
       </c>
       <c r="G10" t="n">
-        <v>27.827</v>
+        <v>9.4582</v>
       </c>
       <c r="H10" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>224</v>
-      </c>
-      <c r="L10" t="n">
-        <v>12</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>ls</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U10" t="n">
-        <v>64</v>
-      </c>
-      <c r="V10" t="inlineStr">
+        <v>12.7651</v>
+      </c>
+      <c r="I10" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="J10" t="n">
+        <v>105.728</v>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>Tesla T4</t>
-        </is>
-      </c>
-      <c r="Y10" t="n">
-        <v>-0.0004</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C03</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="n">
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>swin_tiny</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>224</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10.2475</v>
+      </c>
+      <c r="H11" t="n">
+        <v>11.098</v>
+      </c>
+      <c r="I11" t="n">
+        <v>11.3692</v>
+      </c>
+      <c r="J11" t="n">
+        <v>97.58459999999999</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>224</v>
+      </c>
+      <c r="G12" t="n">
+        <v>7.7865</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="I12" t="n">
+        <v>8.6873</v>
+      </c>
+      <c r="J12" t="n">
+        <v>128.4275</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>efficientnet_b0</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>224</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8.7674</v>
+      </c>
+      <c r="H13" t="n">
+        <v>9.5222</v>
+      </c>
+      <c r="I13" t="n">
+        <v>9.9948</v>
+      </c>
+      <c r="J13" t="n">
+        <v>114.0592</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>mobilenetv3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>224</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5.9894</v>
+      </c>
+      <c r="H14" t="n">
+        <v>6.5658</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6.9726</v>
+      </c>
+      <c r="J14" t="n">
+        <v>166.9619</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>backbone b1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>mobilenetv3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>224</v>
+      </c>
+      <c r="G15" t="n">
+        <v>7.2187</v>
+      </c>
+      <c r="H15" t="n">
+        <v>8.024900000000001</v>
+      </c>
+      <c r="I15" t="n">
+        <v>8.5458</v>
+      </c>
+      <c r="J15" t="n">
+        <v>138.5293</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>I00 1-view 224</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>224</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5.4302</v>
+      </c>
+      <c r="H16" t="n">
+        <v>9.359299999999999</v>
+      </c>
+      <c r="I16" t="n">
+        <v>9.3932</v>
+      </c>
+      <c r="J16" t="n">
+        <v>184.1543</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>I01 flip (K=2) 224</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>224</v>
+      </c>
+      <c r="G17" t="n">
+        <v>8.382999999999999</v>
+      </c>
+      <c r="H17" t="n">
+        <v>11.3782</v>
+      </c>
+      <c r="I17" t="n">
+        <v>11.3972</v>
+      </c>
+      <c r="J17" t="n">
+        <v>238.5771</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>I02b 5crop+flip 192 (K=10)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
         <v>10</v>
       </c>
-      <c r="D11" t="n">
-        <v>0.9655</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.9729</v>
-      </c>
-      <c r="F11" t="n">
-        <v>52.5088</v>
-      </c>
-      <c r="G11" t="n">
-        <v>27.827</v>
-      </c>
-      <c r="H11" t="n">
-        <v>4.4548</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>convnext_tiny</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>in12k_ft_in1k</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
+      <c r="F18" t="n">
+        <v>192</v>
+      </c>
+      <c r="G18" t="n">
+        <v>27.6541</v>
+      </c>
+      <c r="H18" t="n">
+        <v>28.3249</v>
+      </c>
+      <c r="I18" t="n">
+        <v>28.3779</v>
+      </c>
+      <c r="J18" t="n">
+        <v>361.6097</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>I04 res256</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>256</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5.7254</v>
+      </c>
+      <c r="H19" t="n">
+        <v>10.4001</v>
+      </c>
+      <c r="I19" t="n">
+        <v>10.4253</v>
+      </c>
+      <c r="J19" t="n">
+        <v>174.6612</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>I04 res288 (F01)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>288</v>
+      </c>
+      <c r="G20" t="n">
+        <v>6.9092</v>
+      </c>
+      <c r="H20" t="n">
+        <v>9.368499999999999</v>
+      </c>
+      <c r="I20" t="n">
+        <v>9.400399999999999</v>
+      </c>
+      <c r="J20" t="n">
+        <v>144.7347</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>I04 res320</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>320</v>
+      </c>
+      <c r="G21" t="n">
+        <v>8.593500000000001</v>
+      </c>
+      <c r="H21" t="n">
+        <v>14.8999</v>
+      </c>
+      <c r="I21" t="n">
+        <v>14.9273</v>
+      </c>
+      <c r="J21" t="n">
+        <v>116.367</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1-view 224 fp16</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
         <v>224</v>
       </c>
-      <c r="L11" t="n">
-        <v>12</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>finetune</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>color</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>ce</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U11" t="n">
-        <v>64</v>
-      </c>
-      <c r="V11" t="inlineStr">
+      <c r="G22" t="n">
+        <v>5.4245</v>
+      </c>
+      <c r="H22" t="n">
+        <v>5.8617</v>
+      </c>
+      <c r="I22" t="n">
+        <v>6.6243</v>
+      </c>
+      <c r="J22" t="n">
+        <v>184.3481</v>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>2.11.0+cu128</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>1.0.29</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>inference ConvNeXt-T</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1-view 288 fp16</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>Tesla T4</t>
         </is>
       </c>
-      <c r="Y11" t="n">
-        <v>-0.0034</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>288</v>
+      </c>
+      <c r="G23" t="n">
+        <v>5.5909</v>
+      </c>
+      <c r="H23" t="n">
+        <v>5.9172</v>
+      </c>
+      <c r="I23" t="n">
+        <v>6.2062</v>
+      </c>
+      <c r="J23" t="n">
+        <v>178.8613</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>